<commit_message>
Updated variable definitions & set PS legacy check
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/Research/variables/Variable Definitions RQ8_PH2_FEB26.xlsx
+++ b/dashboard-ui/src/components/Research/variables/Variable Definitions RQ8_PH2_FEB26.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\patrick.mohler_cn\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\patrick.mohler_cn\Projects\ITM\itm-evaluation-dashboard\dashboard-ui\src\components\Research\variables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A4E433A-D47B-4836-9BB8-6E113224D043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62122F91-FCD2-4C8B-BBAD-266F3BE991D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1455" yWindow="0" windowWidth="26400" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RQ8" sheetId="1" r:id="rId1"/>
@@ -424,9 +424,6 @@
     <t>Patient A or Patient B</t>
   </si>
   <si>
-    <t>5 = remain in place; 4 = ask for verbal clarification; 3 = attempt to drag patient inside; 2 = express vocal concern but go anyway; 1 = ignore warning</t>
-  </si>
-  <si>
     <t>%</t>
   </si>
   <si>
@@ -535,82 +532,85 @@
     <t>5 = run for cover and wait for all clear; 4 = stop and stare; 3 = attempt to drag patients inside; 2 = express vocal concern but keep treating; 1 = ignore drones</t>
   </si>
   <si>
+    <t>Desert Probe_PS1_Actions</t>
+  </si>
+  <si>
+    <t>Desert Probe_PS2_Actions</t>
+  </si>
+  <si>
+    <t>List of moderator buttons selected in response to initial PS inject</t>
+  </si>
+  <si>
+    <t>List of moderator buttons selected in response to drone</t>
+  </si>
+  <si>
+    <t>Affiliation Focus KDMA measurement from simulation; intercept term (1 of 3 terms in regression approach); TA1 server calculation via probe matcher</t>
+  </si>
+  <si>
+    <t>Affiliation Focus KDMA measurement from OW sim; medical urgency term (2 of 3 terms in regression approach); TA1 server calculation via probe matcher</t>
+  </si>
+  <si>
+    <t>Affiliation Focus KDMA measurement from OW sim; attribute term (3 of 3 terms in regression approach); TA1 server calculation via probe matcher</t>
+  </si>
+  <si>
+    <t>Merit Focus KDMA measurement from OW sim; intercept term (1 of 3 terms in regression approach); TA1 server calculation via probe matcher</t>
+  </si>
+  <si>
+    <t>Merit Focus KDMA measurement from OW sim; medical urgency term (2 of 3 terms in regression approach); TA1 server calculation via probe matcher</t>
+  </si>
+  <si>
+    <t>Merit Focus KDMA measurement from OW sim; attribute term (3 of 3 terms in regression approach); TA1 server calculation via probe matcher</t>
+  </si>
+  <si>
+    <t>Affiliation Focus KDMA measurement from OW sim; medical urgency term (2 of 3 terms in regression approach);TA1 server calculation via probe matcher</t>
+  </si>
+  <si>
+    <t>ADEPT server</t>
+  </si>
+  <si>
+    <t>Alignment between MF_text and MF_urban</t>
+  </si>
+  <si>
+    <t>AF Alignment_Urban</t>
+  </si>
+  <si>
+    <t>MF Alignment_Urban</t>
+  </si>
+  <si>
+    <t>Alignment between AF_text and AF_urban</t>
+  </si>
+  <si>
+    <t>MF Alignment_Desert</t>
+  </si>
+  <si>
+    <t>AF Alignment_Desert</t>
+  </si>
+  <si>
+    <t>Alignment between AF_text and AF_desert</t>
+  </si>
+  <si>
+    <t>Alignment between MF_text and MF_desert</t>
+  </si>
+  <si>
+    <t>Desert Spawn_location</t>
+  </si>
+  <si>
+    <t>Urban Spawn_location</t>
+  </si>
+  <si>
+    <t>The even PIDs (value of 0) spawn inside the big building; the odd PIDs (value of 1) spawn inside the small building.</t>
+  </si>
+  <si>
+    <t>The even PIDs (value of 0) spawn inside the office building; the odd PIDs (value of 1) spawn inside the recycling center.</t>
+  </si>
+  <si>
+    <t>0 or 1</t>
+  </si>
+  <si>
+    <t>4 = Remain in place; 3 = Verbal Response / Ask for clarification; 2 = Drag patient inside; 1 =Ignore warning and approach patient</t>
+  </si>
+  <si>
     <t>5 = remain in place; 4 = verbal concern but remain in place; 3 = attempt to drag patient inside; 2 = express vocal concern but go anyway; 1 = ignore warning</t>
-  </si>
-  <si>
-    <t>Desert Probe_PS1_Actions</t>
-  </si>
-  <si>
-    <t>Desert Probe_PS2_Actions</t>
-  </si>
-  <si>
-    <t>List of moderator buttons selected in response to initial PS inject</t>
-  </si>
-  <si>
-    <t>List of moderator buttons selected in response to drone</t>
-  </si>
-  <si>
-    <t>Affiliation Focus KDMA measurement from simulation; intercept term (1 of 3 terms in regression approach); TA1 server calculation via probe matcher</t>
-  </si>
-  <si>
-    <t>Affiliation Focus KDMA measurement from OW sim; medical urgency term (2 of 3 terms in regression approach); TA1 server calculation via probe matcher</t>
-  </si>
-  <si>
-    <t>Affiliation Focus KDMA measurement from OW sim; attribute term (3 of 3 terms in regression approach); TA1 server calculation via probe matcher</t>
-  </si>
-  <si>
-    <t>Merit Focus KDMA measurement from OW sim; intercept term (1 of 3 terms in regression approach); TA1 server calculation via probe matcher</t>
-  </si>
-  <si>
-    <t>Merit Focus KDMA measurement from OW sim; medical urgency term (2 of 3 terms in regression approach); TA1 server calculation via probe matcher</t>
-  </si>
-  <si>
-    <t>Merit Focus KDMA measurement from OW sim; attribute term (3 of 3 terms in regression approach); TA1 server calculation via probe matcher</t>
-  </si>
-  <si>
-    <t>Affiliation Focus KDMA measurement from OW sim; medical urgency term (2 of 3 terms in regression approach);TA1 server calculation via probe matcher</t>
-  </si>
-  <si>
-    <t>ADEPT server</t>
-  </si>
-  <si>
-    <t>Alignment between MF_text and MF_urban</t>
-  </si>
-  <si>
-    <t>AF Alignment_Urban</t>
-  </si>
-  <si>
-    <t>MF Alignment_Urban</t>
-  </si>
-  <si>
-    <t>Alignment between AF_text and AF_urban</t>
-  </si>
-  <si>
-    <t>MF Alignment_Desert</t>
-  </si>
-  <si>
-    <t>AF Alignment_Desert</t>
-  </si>
-  <si>
-    <t>Alignment between AF_text and AF_desert</t>
-  </si>
-  <si>
-    <t>Alignment between MF_text and MF_desert</t>
-  </si>
-  <si>
-    <t>Desert Spawn_location</t>
-  </si>
-  <si>
-    <t>Urban Spawn_location</t>
-  </si>
-  <si>
-    <t>The even PIDs (value of 0) spawn inside the big building; the odd PIDs (value of 1) spawn inside the small building.</t>
-  </si>
-  <si>
-    <t>The even PIDs (value of 0) spawn inside the office building; the odd PIDs (value of 1) spawn inside the recycling center.</t>
-  </si>
-  <si>
-    <t>0 or 1</t>
   </si>
 </sst>
 </file>
@@ -1149,10 +1149,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F1" s="19" t="s">
         <v>3</v>
@@ -1185,10 +1185,10 @@
         <v>12</v>
       </c>
       <c r="P1" s="19" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="Q1" s="19" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="R1" s="17" t="s">
         <v>13</v>
@@ -1398,16 +1398,16 @@
         <v>81</v>
       </c>
       <c r="CI1" s="12" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="CJ1" s="12" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="CK1" s="12" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="CL1" s="12" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:90" s="7" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
@@ -1670,16 +1670,16 @@
         <v>87</v>
       </c>
       <c r="CI2" s="12" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="CJ2" s="12" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="CK2" s="12" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="CL2" s="12" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:90" s="7" customFormat="1" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1693,10 +1693,10 @@
         <v>90</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F3" s="19" t="s">
         <v>91</v>
@@ -1726,13 +1726,13 @@
         <v>93</v>
       </c>
       <c r="O3" s="19" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="P3" s="19" t="s">
         <v>93</v>
       </c>
       <c r="Q3" s="19" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="R3" s="17" t="s">
         <v>94</v>
@@ -1906,52 +1906,52 @@
         <v>124</v>
       </c>
       <c r="BW3" s="24" t="s">
+        <v>168</v>
+      </c>
+      <c r="BX3" s="24" t="s">
+        <v>169</v>
+      </c>
+      <c r="BY3" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="BX3" s="24" t="s">
+      <c r="BZ3" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="BY3" s="24" t="s">
+      <c r="CA3" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="BZ3" s="24" t="s">
+      <c r="CB3" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="CA3" s="24" t="s">
+      <c r="CC3" s="24" t="s">
+        <v>168</v>
+      </c>
+      <c r="CD3" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="CB3" s="24" t="s">
-        <v>175</v>
-      </c>
-      <c r="CC3" s="24" t="s">
+      <c r="CE3" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="CD3" s="24" t="s">
+      <c r="CF3" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="CG3" s="24" t="s">
+        <v>172</v>
+      </c>
+      <c r="CH3" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="CI3" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="CJ3" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="CK3" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="CE3" s="24" t="s">
-        <v>172</v>
-      </c>
-      <c r="CF3" s="24" t="s">
-        <v>173</v>
-      </c>
-      <c r="CG3" s="24" t="s">
-        <v>174</v>
-      </c>
-      <c r="CH3" s="24" t="s">
-        <v>175</v>
-      </c>
-      <c r="CI3" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="CJ3" s="12" t="s">
-        <v>184</v>
-      </c>
-      <c r="CK3" s="12" t="s">
-        <v>178</v>
-      </c>
       <c r="CL3" s="12" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:90" s="7" customFormat="1" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1963,10 +1963,10 @@
         <v>126</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F4" s="19" t="s">
         <v>127</v>
@@ -1993,16 +1993,16 @@
         <v>127</v>
       </c>
       <c r="N4" s="19" t="s">
-        <v>165</v>
+        <v>190</v>
       </c>
       <c r="O4" s="19" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="P4" s="19" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="Q4" s="19" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="R4" s="17" t="s">
         <v>127</v>
@@ -2029,115 +2029,115 @@
         <v>127</v>
       </c>
       <c r="Z4" s="17" t="s">
+        <v>189</v>
+      </c>
+      <c r="AA4" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="AA4" s="19" t="s">
+      <c r="AB4" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="AB4" s="19" t="s">
+      <c r="AC4" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="AC4" s="19" t="s">
+      <c r="AD4" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="AE4" s="17" t="s">
+        <v>129</v>
+      </c>
+      <c r="AF4" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="AG4" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="AD4" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="AE4" s="17" t="s">
+      <c r="AH4" s="19" t="s">
+        <v>131</v>
+      </c>
+      <c r="AI4" s="19" t="s">
+        <v>131</v>
+      </c>
+      <c r="AJ4" s="19" t="s">
+        <v>131</v>
+      </c>
+      <c r="AK4" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="AF4" s="17" t="s">
+      <c r="AL4" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="AM4" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="AG4" s="19" t="s">
+      <c r="AN4" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="AH4" s="19" t="s">
+      <c r="AO4" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="AP4" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="AQ4" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="AR4" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="AS4" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="AT4" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="AU4" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="AV4" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="AW4" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="AI4" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="AJ4" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="AK4" s="19" t="s">
+      <c r="AX4" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="AY4" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="AZ4" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="AL4" s="19" t="s">
+      <c r="BA4" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="BB4" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="AM4" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="AN4" s="19" t="s">
+      <c r="BC4" s="19" t="s">
+        <v>131</v>
+      </c>
+      <c r="BD4" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="BE4" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="BF4" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="BG4" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="AO4" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="AP4" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="AQ4" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="AR4" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="AS4" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="AT4" s="17" t="s">
+      <c r="BH4" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="AU4" s="17" t="s">
+      <c r="BI4" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="AV4" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="AW4" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="AX4" s="17" t="s">
-        <v>134</v>
-      </c>
-      <c r="AY4" s="19" t="s">
+      <c r="BJ4" s="17" t="s">
         <v>135</v>
-      </c>
-      <c r="AZ4" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="BA4" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="BB4" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="BC4" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="BD4" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="BE4" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="BF4" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="BG4" s="17" t="s">
-        <v>134</v>
-      </c>
-      <c r="BH4" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="BI4" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="BJ4" s="17" t="s">
-        <v>136</v>
       </c>
       <c r="BK4" s="15"/>
       <c r="BL4" s="15"/>
@@ -2243,136 +2243,136 @@
   <sheetData>
     <row r="1" spans="1:6" s="11" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="C1" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="9" t="s">
         <v>141</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>146</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>147</v>
       </c>
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>156</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>156</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="2"/>
@@ -10329,136 +10329,136 @@
   <sheetData>
     <row r="1" spans="1:6" s="11" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="C1" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="9" t="s">
         <v>141</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>145</v>
-      </c>
       <c r="E2" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="2"/>

</xml_diff>

<commit_message>
Updated variable definition for evac & dragged
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/Research/variables/Variable Definitions RQ8_PH2_FEB26.xlsx
+++ b/dashboard-ui/src/components/Research/variables/Variable Definitions RQ8_PH2_FEB26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\patrick.mohler_cn\Projects\ITM\itm-evaluation-dashboard\dashboard-ui\src\components\Research\variables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62122F91-FCD2-4C8B-BBAD-266F3BE991D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E843824C-3A63-40FC-B31C-C6622C163E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1455" yWindow="0" windowWidth="26400" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RQ8" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="196">
   <si>
     <t>Variables</t>
   </si>
@@ -611,6 +611,21 @@
   </si>
   <si>
     <t>5 = remain in place; 4 = verbal concern but remain in place; 3 = attempt to drag patient inside; 2 = express vocal concern but go anyway; 1 = ignore warning</t>
+  </si>
+  <si>
+    <t>Desert Patient{N}_dragged</t>
+  </si>
+  <si>
+    <t>Whether patient {N} was dragged at any point or not</t>
+  </si>
+  <si>
+    <t>Yes/No</t>
+  </si>
+  <si>
+    <t>Urban Patient{N}_dragged</t>
+  </si>
+  <si>
+    <t>0 = No evac, 1 = Round 1 evac, 2 = Round 2 evac</t>
   </si>
 </sst>
 </file>
@@ -1096,7 +1111,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:CL6"/>
+  <dimension ref="A1:CN6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="16.7109375" style="6" bestFit="1" customWidth="1"/>
@@ -1114,31 +1129,31 @@
     <col min="37" max="41" width="13" style="20" bestFit="1" customWidth="1"/>
     <col min="42" max="45" width="16.7109375" style="18" bestFit="1" customWidth="1"/>
     <col min="46" max="50" width="13" style="18" bestFit="1" customWidth="1"/>
-    <col min="51" max="56" width="13" style="20" bestFit="1" customWidth="1"/>
-    <col min="57" max="62" width="13" style="18" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="87.7109375" style="16" customWidth="1"/>
-    <col min="64" max="65" width="73" style="16" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="38.5703125" style="14" customWidth="1"/>
-    <col min="67" max="67" width="34.7109375" style="14" customWidth="1"/>
-    <col min="68" max="68" width="73" style="16" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="32.5703125" style="14" customWidth="1"/>
-    <col min="70" max="74" width="32.28515625" style="14" customWidth="1"/>
-    <col min="75" max="75" width="87.7109375" style="25" customWidth="1"/>
-    <col min="76" max="77" width="73" style="25" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="38.5703125" style="23" customWidth="1"/>
-    <col min="79" max="79" width="34.7109375" style="23" customWidth="1"/>
-    <col min="80" max="80" width="73" style="25" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="87.7109375" style="25" customWidth="1"/>
-    <col min="82" max="83" width="73" style="25" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="38.5703125" style="23" customWidth="1"/>
-    <col min="85" max="85" width="34.7109375" style="23" customWidth="1"/>
-    <col min="86" max="86" width="73" style="25" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="14.7109375" style="13" customWidth="1"/>
-    <col min="88" max="88" width="15.28515625" style="13" customWidth="1"/>
-    <col min="89" max="90" width="9.140625" style="13"/>
+    <col min="51" max="57" width="13" style="20" bestFit="1" customWidth="1"/>
+    <col min="58" max="64" width="13" style="18" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="87.7109375" style="16" customWidth="1"/>
+    <col min="66" max="67" width="73" style="16" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="38.5703125" style="14" customWidth="1"/>
+    <col min="69" max="69" width="34.7109375" style="14" customWidth="1"/>
+    <col min="70" max="70" width="73" style="16" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="32.5703125" style="14" customWidth="1"/>
+    <col min="72" max="76" width="32.28515625" style="14" customWidth="1"/>
+    <col min="77" max="77" width="87.7109375" style="25" customWidth="1"/>
+    <col min="78" max="79" width="73" style="25" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="38.5703125" style="23" customWidth="1"/>
+    <col min="81" max="81" width="34.7109375" style="23" customWidth="1"/>
+    <col min="82" max="82" width="73" style="25" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="87.7109375" style="25" customWidth="1"/>
+    <col min="84" max="85" width="73" style="25" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="38.5703125" style="23" customWidth="1"/>
+    <col min="87" max="87" width="34.7109375" style="23" customWidth="1"/>
+    <col min="88" max="88" width="73" style="25" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="14.7109375" style="13" customWidth="1"/>
+    <col min="90" max="90" width="15.28515625" style="13" customWidth="1"/>
+    <col min="91" max="92" width="9.140625" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:90" s="7" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:92" s="7" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1307,110 +1322,116 @@
       <c r="BD1" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="BE1" s="17" t="s">
+      <c r="BE1" s="19" t="s">
+        <v>191</v>
+      </c>
+      <c r="BF1" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="BF1" s="17" t="s">
+      <c r="BG1" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="BG1" s="17" t="s">
+      <c r="BH1" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="BH1" s="17" t="s">
+      <c r="BI1" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="BI1" s="17" t="s">
+      <c r="BJ1" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="BJ1" s="17" t="s">
+      <c r="BK1" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="BK1" s="14" t="s">
+      <c r="BL1" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="BM1" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="BL1" s="14" t="s">
+      <c r="BN1" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="BM1" s="14" t="s">
+      <c r="BO1" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="BN1" s="14" t="s">
+      <c r="BP1" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="BO1" s="14" t="s">
+      <c r="BQ1" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="BP1" s="14" t="s">
+      <c r="BR1" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="BQ1" s="14" t="s">
+      <c r="BS1" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="BR1" s="14" t="s">
+      <c r="BT1" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="BS1" s="14" t="s">
+      <c r="BU1" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="BT1" s="14" t="s">
+      <c r="BV1" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="BU1" s="14" t="s">
+      <c r="BW1" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="BV1" s="14" t="s">
+      <c r="BX1" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="BW1" s="23" t="s">
+      <c r="BY1" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="BX1" s="23" t="s">
+      <c r="BZ1" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="BY1" s="23" t="s">
+      <c r="CA1" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="BZ1" s="23" t="s">
+      <c r="CB1" s="23" t="s">
         <v>73</v>
       </c>
-      <c r="CA1" s="23" t="s">
+      <c r="CC1" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="CB1" s="23" t="s">
+      <c r="CD1" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="CC1" s="23" t="s">
+      <c r="CE1" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="CD1" s="23" t="s">
+      <c r="CF1" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="CE1" s="23" t="s">
+      <c r="CG1" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="CF1" s="23" t="s">
+      <c r="CH1" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="CG1" s="23" t="s">
+      <c r="CI1" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="CH1" s="23" t="s">
+      <c r="CJ1" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="CI1" s="12" t="s">
+      <c r="CK1" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="CJ1" s="12" t="s">
+      <c r="CL1" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="CK1" s="12" t="s">
+      <c r="CM1" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="CL1" s="12" t="s">
+      <c r="CN1" s="12" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="2" spans="1:90" s="7" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:92" s="7" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>82</v>
       </c>
@@ -1579,7 +1600,7 @@
       <c r="BD2" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="BE2" s="17" t="s">
+      <c r="BE2" s="19" t="s">
         <v>85</v>
       </c>
       <c r="BF2" s="17" t="s">
@@ -1597,11 +1618,11 @@
       <c r="BJ2" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="BK2" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="BL2" s="15" t="s">
-        <v>86</v>
+      <c r="BK2" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="BL2" s="17" t="s">
+        <v>85</v>
       </c>
       <c r="BM2" s="15" t="s">
         <v>86</v>
@@ -1633,11 +1654,11 @@
       <c r="BV2" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="BW2" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="BX2" s="24" t="s">
-        <v>87</v>
+      <c r="BW2" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="BX2" s="15" t="s">
+        <v>86</v>
       </c>
       <c r="BY2" s="24" t="s">
         <v>87</v>
@@ -1669,11 +1690,11 @@
       <c r="CH2" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="CI2" s="12" t="s">
-        <v>175</v>
-      </c>
-      <c r="CJ2" s="12" t="s">
-        <v>175</v>
+      <c r="CI2" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="CJ2" s="24" t="s">
+        <v>87</v>
       </c>
       <c r="CK2" s="12" t="s">
         <v>175</v>
@@ -1681,8 +1702,14 @@
       <c r="CL2" s="12" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="3" spans="1:90" s="7" customFormat="1" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CM2" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="CN2" s="12" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="3" spans="1:92" s="7" customFormat="1" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>88</v>
       </c>
@@ -1851,110 +1878,116 @@
       <c r="BD3" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="BE3" s="17" t="s">
+      <c r="BE3" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="BF3" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="BF3" s="17" t="s">
+      <c r="BG3" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="BG3" s="17" t="s">
+      <c r="BH3" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="BH3" s="17" t="s">
+      <c r="BI3" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="BI3" s="17" t="s">
+      <c r="BJ3" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="BJ3" s="17" t="s">
+      <c r="BK3" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="BK3" s="15" t="s">
+      <c r="BL3" s="17" t="s">
+        <v>192</v>
+      </c>
+      <c r="BM3" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="BL3" s="15" t="s">
+      <c r="BN3" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="BM3" s="15" t="s">
+      <c r="BO3" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="BN3" s="15" t="s">
+      <c r="BP3" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="BO3" s="15" t="s">
+      <c r="BQ3" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="BP3" s="15" t="s">
+      <c r="BR3" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="BQ3" s="15" t="s">
+      <c r="BS3" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="BR3" s="15" t="s">
+      <c r="BT3" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="BS3" s="15" t="s">
+      <c r="BU3" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="BT3" s="15" t="s">
+      <c r="BV3" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="BU3" s="15" t="s">
+      <c r="BW3" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="BV3" s="15" t="s">
+      <c r="BX3" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="BW3" s="24" t="s">
+      <c r="BY3" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="BX3" s="24" t="s">
+      <c r="BZ3" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="BY3" s="24" t="s">
+      <c r="CA3" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="BZ3" s="24" t="s">
+      <c r="CB3" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="CA3" s="24" t="s">
+      <c r="CC3" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="CB3" s="24" t="s">
+      <c r="CD3" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="CC3" s="24" t="s">
+      <c r="CE3" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="CD3" s="24" t="s">
+      <c r="CF3" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="CE3" s="24" t="s">
+      <c r="CG3" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="CF3" s="24" t="s">
+      <c r="CH3" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="CG3" s="24" t="s">
+      <c r="CI3" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="CH3" s="24" t="s">
+      <c r="CJ3" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="CI3" s="12" t="s">
+      <c r="CK3" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="CJ3" s="12" t="s">
+      <c r="CL3" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="CK3" s="12" t="s">
+      <c r="CM3" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="CL3" s="12" t="s">
+      <c r="CN3" s="12" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="4" spans="1:90" s="7" customFormat="1" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:92" s="7" customFormat="1" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>125</v>
       </c>
@@ -2110,7 +2143,7 @@
         <v>131</v>
       </c>
       <c r="BA4" s="19" t="s">
-        <v>133</v>
+        <v>195</v>
       </c>
       <c r="BB4" s="19" t="s">
         <v>131</v>
@@ -2121,26 +2154,30 @@
       <c r="BD4" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="BE4" s="17" t="s">
+      <c r="BE4" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="BF4" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="BF4" s="17" t="s">
+      <c r="BG4" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="BG4" s="17" t="s">
-        <v>133</v>
-      </c>
       <c r="BH4" s="17" t="s">
-        <v>131</v>
+        <v>195</v>
       </c>
       <c r="BI4" s="17" t="s">
         <v>131</v>
       </c>
       <c r="BJ4" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="BK4" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="BK4" s="15"/>
-      <c r="BL4" s="15"/>
+      <c r="BL4" s="17" t="s">
+        <v>193</v>
+      </c>
       <c r="BM4" s="15"/>
       <c r="BN4" s="15"/>
       <c r="BO4" s="15"/>
@@ -2151,8 +2188,8 @@
       <c r="BT4" s="15"/>
       <c r="BU4" s="15"/>
       <c r="BV4" s="15"/>
-      <c r="BW4" s="24"/>
-      <c r="BX4" s="24"/>
+      <c r="BW4" s="15"/>
+      <c r="BX4" s="15"/>
       <c r="BY4" s="24"/>
       <c r="BZ4" s="24"/>
       <c r="CA4" s="24"/>
@@ -2163,14 +2200,14 @@
       <c r="CF4" s="24"/>
       <c r="CG4" s="24"/>
       <c r="CH4" s="24"/>
-      <c r="CI4" s="12"/>
-      <c r="CJ4" s="12"/>
+      <c r="CI4" s="24"/>
+      <c r="CJ4" s="24"/>
       <c r="CK4" s="12"/>
       <c r="CL4" s="12"/>
-    </row>
-    <row r="5" spans="1:90" x14ac:dyDescent="0.25">
-      <c r="BK5" s="15"/>
-      <c r="BL5" s="15"/>
+      <c r="CM4" s="12"/>
+      <c r="CN4" s="12"/>
+    </row>
+    <row r="5" spans="1:92" x14ac:dyDescent="0.25">
       <c r="BM5" s="15"/>
       <c r="BN5" s="15"/>
       <c r="BO5" s="15"/>
@@ -2181,8 +2218,8 @@
       <c r="BT5" s="15"/>
       <c r="BU5" s="15"/>
       <c r="BV5" s="15"/>
-      <c r="BW5" s="24"/>
-      <c r="BX5" s="24"/>
+      <c r="BW5" s="15"/>
+      <c r="BX5" s="15"/>
       <c r="BY5" s="24"/>
       <c r="BZ5" s="24"/>
       <c r="CA5" s="24"/>
@@ -2193,10 +2230,10 @@
       <c r="CF5" s="24"/>
       <c r="CG5" s="24"/>
       <c r="CH5" s="24"/>
-    </row>
-    <row r="6" spans="1:90" x14ac:dyDescent="0.25">
-      <c r="BK6" s="15"/>
-      <c r="BL6" s="15"/>
+      <c r="CI5" s="24"/>
+      <c r="CJ5" s="24"/>
+    </row>
+    <row r="6" spans="1:92" x14ac:dyDescent="0.25">
       <c r="BM6" s="15"/>
       <c r="BN6" s="15"/>
       <c r="BO6" s="15"/>
@@ -2207,8 +2244,8 @@
       <c r="BT6" s="15"/>
       <c r="BU6" s="15"/>
       <c r="BV6" s="15"/>
-      <c r="BW6" s="24"/>
-      <c r="BX6" s="24"/>
+      <c r="BW6" s="15"/>
+      <c r="BX6" s="15"/>
       <c r="BY6" s="24"/>
       <c r="BZ6" s="24"/>
       <c r="CA6" s="24"/>
@@ -2219,6 +2256,8 @@
       <c r="CF6" s="24"/>
       <c r="CG6" s="24"/>
       <c r="CH6" s="24"/>
+      <c r="CI6" s="24"/>
+      <c r="CJ6" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>